<commit_message>
add documentation for phisical components
</commit_message>
<xml_diff>
--- a/workspaces/traject_224/input/input.xlsx
+++ b/workspaces/traject_224/input/input.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\CP\git_clones\GeoProb-Pipe\GeoProb-PipeV2\GeoProb-Pipe\workspaces\traject_224\input\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://wsrlnl-my.sharepoint.com/personal/s_kapinga_wsrl_nl/Documents/Documenten/Github/GeoProb-Pipe/workspaces/traject_224/input/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:20001_{2E794C68-BC23-489F-99A1-881B494B69FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="2" documentId="13_ncr:20001_{2E794C68-BC23-489F-99A1-881B494B69FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9DF22BBC-5B82-5B60-8663-DEB1960CD597}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{E14FA4F5-43AA-4DAE-BCE2-7688F4F5853B}"/>
   </bookViews>
@@ -20,7 +20,6 @@
     <sheet name="Settings" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>

</xml_diff>

<commit_message>
Controle en sanity check op input. Bij een vak een tussenzandscenario toegevoegd
</commit_message>
<xml_diff>
--- a/workspaces/traject_224/input/input.xlsx
+++ b/workspaces/traject_224/input/input.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://wsrlnl-my.sharepoint.com/personal/s_kapinga_wsrl_nl/Documents/Documenten/Github/GeoProb-Pipe/workspaces/traject_224/input/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2" documentId="13_ncr:20001_{2E794C68-BC23-489F-99A1-881B494B69FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9DF22BBC-5B82-5B60-8663-DEB1960CD597}"/>
+  <xr:revisionPtr revIDLastSave="58" documentId="13_ncr:20001_{2E794C68-BC23-489F-99A1-881B494B69FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7DB16BF9-EF35-4B1F-99F3-10D1310B1015}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{E14FA4F5-43AA-4DAE-BCE2-7688F4F5853B}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{E14FA4F5-43AA-4DAE-BCE2-7688F4F5853B}"/>
   </bookViews>
   <sheets>
     <sheet name="Vakken" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="573" uniqueCount="224">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="574" uniqueCount="225">
   <si>
     <t>M_van</t>
   </si>
@@ -712,6 +712,9 @@
   </si>
   <si>
     <t>HA063.+074-RK000.+005</t>
+  </si>
+  <si>
+    <t>TZ</t>
   </si>
 </sst>
 </file>
@@ -808,7 +811,7 @@
     <cellStyle name="Normal 2" xfId="1" xr:uid="{11010186-4FF4-48E2-AD4E-93BC10A29908}"/>
     <cellStyle name="Standaard" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="11">
+  <dxfs count="12">
     <dxf>
       <fill>
         <patternFill>
@@ -856,6 +859,9 @@
       <numFmt numFmtId="15" formatCode="0.00E+00"/>
     </dxf>
     <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
       <numFmt numFmtId="2" formatCode="0.00"/>
     </dxf>
   </dxfs>
@@ -885,7 +891,7 @@
     <tableColumn id="9" xr3:uid="{C7E61DAC-831F-4734-9A0F-D17FA66D5C5C}" name="Kolom9"/>
     <tableColumn id="10" xr3:uid="{DC962EDF-740C-439F-836D-211E1F74A71C}" name="Kolom10"/>
     <tableColumn id="11" xr3:uid="{2DF82AEB-01BF-44F4-BB8B-81DDACEA5D0F}" name="Kolom11"/>
-    <tableColumn id="13" xr3:uid="{D266588F-C618-4806-A218-A5D90FF4D5E3}" name="Kolom13" dataDxfId="10"/>
+    <tableColumn id="13" xr3:uid="{D266588F-C618-4806-A218-A5D90FF4D5E3}" name="Kolom13" dataDxfId="11"/>
     <tableColumn id="14" xr3:uid="{C17CFC23-4C11-4C47-AEE5-4FB4BCCD1A66}" name="Kolom14"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -893,7 +899,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{9844274D-7B34-420F-9662-89C5C9A298BD}" name="Tabel10" displayName="Tabel10" ref="A2:P15" headerRowCount="0" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{9844274D-7B34-420F-9662-89C5C9A298BD}" name="Tabel10" displayName="Tabel10" ref="A2:P16" headerRowCount="0" totalsRowShown="0">
   <tableColumns count="16">
     <tableColumn id="2" xr3:uid="{E80206AD-C5FD-4475-B5E4-08A08DA66E4A}" name="Kolom2"/>
     <tableColumn id="13" xr3:uid="{39F38892-EB92-4E2D-A4CE-461B1DC8B27E}" name="Column1"/>
@@ -902,7 +908,9 @@
     <tableColumn id="5" xr3:uid="{D8D86CD9-C3BF-42A4-A962-B1DB26AE3B59}" name="Kolom5"/>
     <tableColumn id="6" xr3:uid="{7BE88CD6-31E3-4118-B387-294A1FF1B8B4}" name="Kolom6"/>
     <tableColumn id="7" xr3:uid="{6C73C0C2-7F10-4F3F-8B62-E3B2A460FC52}" name="Kolom7"/>
-    <tableColumn id="8" xr3:uid="{44A8D682-C1F2-412E-9F5A-3E4254057E71}" name="Kolom8"/>
+    <tableColumn id="8" xr3:uid="{44A8D682-C1F2-412E-9F5A-3E4254057E71}" name="Kolom8" dataDxfId="10">
+      <calculatedColumnFormula>0.05*Tabel10[[#This Row],[Kolom7]]</calculatedColumnFormula>
+    </tableColumn>
     <tableColumn id="9" xr3:uid="{DE4A1EC2-2C76-4840-9AF4-87A3533169E8}" name="Kolom9"/>
     <tableColumn id="10" xr3:uid="{30E95029-7E84-4404-97EA-CC899B222DC3}" name="Kolom10"/>
     <tableColumn id="11" xr3:uid="{21D2E504-CBB5-45F7-9119-E1DA7B53C2D5}" name="Kolom11"/>
@@ -1270,7 +1278,7 @@
     <col min="5" max="5" width="16.625" customWidth="1"/>
     <col min="6" max="6" width="18.25" customWidth="1"/>
     <col min="7" max="7" width="11.125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="15" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="16.125" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="17.375" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1301,7 +1309,7 @@
       </c>
       <c r="I1" s="9" t="str">
         <f>LEFT(H1,LEN(H1)-5)&amp;VLOOKUP(LEFT(H1,LEN(H1)-5),Overzicht_parameters!$A$2:$F$69,6,(FALSE))</f>
-        <v>c_voorland_stdev</v>
+        <v>c_voorland_vc</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.15">
@@ -3584,7 +3592,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A3ED9FF6-8968-4FA6-BAEC-B95365AA2886}">
-  <dimension ref="A1:P15"/>
+  <dimension ref="A1:P16"/>
   <sheetFormatPr defaultRowHeight="11.25" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="1" max="1" width="20.75" bestFit="1" customWidth="1"/>
@@ -3669,7 +3677,7 @@
         <v>17</v>
       </c>
       <c r="D2">
-        <v>0.5</v>
+        <v>0.25</v>
       </c>
       <c r="E2">
         <v>1</v>
@@ -3678,10 +3686,11 @@
         <v>0.5</v>
       </c>
       <c r="G2">
-        <v>18.5</v>
+        <v>16.5</v>
       </c>
       <c r="H2">
-        <v>0.92500000000000004</v>
+        <f>0.05*Tabel10[[#This Row],[Kolom7]]</f>
+        <v>0.82500000000000007</v>
       </c>
       <c r="I2">
         <v>10.5</v>
@@ -3719,18 +3728,19 @@
         <v>18</v>
       </c>
       <c r="D3">
-        <v>0.5</v>
+        <v>0.75</v>
       </c>
       <c r="E3">
-        <v>-0.5</v>
+        <v>1.8</v>
       </c>
       <c r="F3">
-        <v>0.5</v>
+        <v>0.3</v>
       </c>
       <c r="G3">
         <v>18.5</v>
       </c>
       <c r="H3">
+        <f>0.05*Tabel10[[#This Row],[Kolom7]]</f>
         <v>0.92500000000000004</v>
       </c>
       <c r="I3">
@@ -3746,7 +3756,7 @@
         <v>0.35</v>
       </c>
       <c r="M3" s="1">
-        <v>4.4999999999999999E-4</v>
+        <v>3.5E-4</v>
       </c>
       <c r="N3">
         <v>0.12</v>
@@ -3760,7 +3770,7 @@
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.15">
       <c r="A4">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="B4">
         <v>0</v>
@@ -3778,10 +3788,11 @@
         <v>0.5</v>
       </c>
       <c r="G4">
-        <v>18.5</v>
+        <v>16.5</v>
       </c>
       <c r="H4">
-        <v>0.92500000000000004</v>
+        <f>0.05*Tabel10[[#This Row],[Kolom7]]</f>
+        <v>0.82500000000000007</v>
       </c>
       <c r="I4">
         <v>10.5</v>
@@ -3810,7 +3821,7 @@
     </row>
     <row r="5" spans="1:16" x14ac:dyDescent="0.15">
       <c r="A5">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="B5">
         <v>0</v>
@@ -3822,15 +3833,16 @@
         <v>0.5</v>
       </c>
       <c r="E5">
-        <v>-0.5</v>
+        <v>2</v>
       </c>
       <c r="F5">
-        <v>0.5</v>
+        <v>0.3</v>
       </c>
       <c r="G5">
         <v>18.5</v>
       </c>
       <c r="H5">
+        <f>0.05*Tabel10[[#This Row],[Kolom7]]</f>
         <v>0.92500000000000004</v>
       </c>
       <c r="I5">
@@ -3860,7 +3872,7 @@
     </row>
     <row r="6" spans="1:16" x14ac:dyDescent="0.15">
       <c r="A6">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="B6">
         <v>1</v>
@@ -3878,10 +3890,11 @@
         <v>0.5</v>
       </c>
       <c r="G6">
-        <v>18.5</v>
+        <v>16.5</v>
       </c>
       <c r="H6">
-        <v>0.92500000000000004</v>
+        <f>0.05*Tabel10[[#This Row],[Kolom7]]</f>
+        <v>0.82500000000000007</v>
       </c>
       <c r="I6">
         <v>10.5</v>
@@ -3910,7 +3923,7 @@
     </row>
     <row r="7" spans="1:16" x14ac:dyDescent="0.15">
       <c r="A7">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="B7">
         <v>1</v>
@@ -3922,15 +3935,16 @@
         <v>0.5</v>
       </c>
       <c r="E7">
-        <v>-0.5</v>
+        <v>1.5</v>
       </c>
       <c r="F7">
-        <v>0.5</v>
+        <v>0.3</v>
       </c>
       <c r="G7">
         <v>18.5</v>
       </c>
       <c r="H7">
+        <f>0.05*Tabel10[[#This Row],[Kolom7]]</f>
         <v>0.92500000000000004</v>
       </c>
       <c r="I7">
@@ -3960,7 +3974,7 @@
     </row>
     <row r="8" spans="1:16" x14ac:dyDescent="0.15">
       <c r="A8">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="B8">
         <v>2</v>
@@ -3978,10 +3992,11 @@
         <v>0.5</v>
       </c>
       <c r="G8">
-        <v>18.5</v>
+        <v>16.5</v>
       </c>
       <c r="H8">
-        <v>0.92500000000000004</v>
+        <f>0.05*Tabel10[[#This Row],[Kolom7]]</f>
+        <v>0.82500000000000007</v>
       </c>
       <c r="I8">
         <v>10.5</v>
@@ -4010,7 +4025,7 @@
     </row>
     <row r="9" spans="1:16" x14ac:dyDescent="0.15">
       <c r="A9">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="B9">
         <v>2</v>
@@ -4022,15 +4037,16 @@
         <v>0.5</v>
       </c>
       <c r="E9">
-        <v>-0.5</v>
+        <v>2.2000000000000002</v>
       </c>
       <c r="F9">
-        <v>0.5</v>
+        <v>0.3</v>
       </c>
       <c r="G9">
         <v>18.5</v>
       </c>
       <c r="H9">
+        <f>0.05*Tabel10[[#This Row],[Kolom7]]</f>
         <v>0.92500000000000004</v>
       </c>
       <c r="I9">
@@ -4060,7 +4076,7 @@
     </row>
     <row r="10" spans="1:16" x14ac:dyDescent="0.15">
       <c r="A10">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="B10">
         <v>3</v>
@@ -4078,10 +4094,11 @@
         <v>0.5</v>
       </c>
       <c r="G10">
-        <v>18.5</v>
+        <v>16.5</v>
       </c>
       <c r="H10">
-        <v>0.92500000000000004</v>
+        <f>0.05*Tabel10[[#This Row],[Kolom7]]</f>
+        <v>0.82500000000000007</v>
       </c>
       <c r="I10">
         <v>10.5</v>
@@ -4110,7 +4127,7 @@
     </row>
     <row r="11" spans="1:16" x14ac:dyDescent="0.15">
       <c r="A11">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="B11">
         <v>3</v>
@@ -4122,15 +4139,16 @@
         <v>0.5</v>
       </c>
       <c r="E11">
-        <v>-0.5</v>
+        <v>1.5</v>
       </c>
       <c r="F11">
-        <v>0.5</v>
+        <v>0.3</v>
       </c>
       <c r="G11">
         <v>18.5</v>
       </c>
       <c r="H11">
+        <f>0.05*Tabel10[[#This Row],[Kolom7]]</f>
         <v>0.92500000000000004</v>
       </c>
       <c r="I11">
@@ -4160,7 +4178,7 @@
     </row>
     <row r="12" spans="1:16" x14ac:dyDescent="0.15">
       <c r="A12">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="B12">
         <v>4</v>
@@ -4172,16 +4190,17 @@
         <v>0.5</v>
       </c>
       <c r="E12">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="F12">
         <v>0.5</v>
       </c>
       <c r="G12">
-        <v>18.5</v>
+        <v>16.5</v>
       </c>
       <c r="H12">
-        <v>0.92500000000000004</v>
+        <f>0.05*Tabel10[[#This Row],[Kolom7]]</f>
+        <v>0.82500000000000007</v>
       </c>
       <c r="I12">
         <v>10.5</v>
@@ -4210,7 +4229,7 @@
     </row>
     <row r="13" spans="1:16" x14ac:dyDescent="0.15">
       <c r="A13">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="B13">
         <v>4</v>
@@ -4222,15 +4241,16 @@
         <v>0.5</v>
       </c>
       <c r="E13">
-        <v>-0.5</v>
+        <v>1.2</v>
       </c>
       <c r="F13">
-        <v>0.5</v>
+        <v>0.3</v>
       </c>
       <c r="G13">
         <v>18.5</v>
       </c>
       <c r="H13">
+        <f>0.05*Tabel10[[#This Row],[Kolom7]]</f>
         <v>0.92500000000000004</v>
       </c>
       <c r="I13">
@@ -4260,7 +4280,7 @@
     </row>
     <row r="14" spans="1:16" x14ac:dyDescent="0.15">
       <c r="A14">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B14">
         <v>5</v>
@@ -4269,19 +4289,20 @@
         <v>17</v>
       </c>
       <c r="D14">
-        <v>0.5</v>
+        <v>0.3</v>
       </c>
       <c r="E14">
-        <v>1</v>
+        <v>-3</v>
       </c>
       <c r="F14">
         <v>0.5</v>
       </c>
       <c r="G14">
-        <v>18.5</v>
+        <v>16.5</v>
       </c>
       <c r="H14">
-        <v>0.92500000000000004</v>
+        <f>0.05*Tabel10[[#This Row],[Kolom7]]</f>
+        <v>0.82500000000000007</v>
       </c>
       <c r="I14">
         <v>10.5</v>
@@ -4310,7 +4331,7 @@
     </row>
     <row r="15" spans="1:16" x14ac:dyDescent="0.15">
       <c r="A15">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B15">
         <v>5</v>
@@ -4319,18 +4340,19 @@
         <v>18</v>
       </c>
       <c r="D15">
-        <v>0.5</v>
+        <v>0.4</v>
       </c>
       <c r="E15">
-        <v>-0.5</v>
+        <v>2.5</v>
       </c>
       <c r="F15">
-        <v>0.5</v>
+        <v>0.3</v>
       </c>
       <c r="G15">
         <v>18.5</v>
       </c>
       <c r="H15">
+        <f>0.05*Tabel10[[#This Row],[Kolom7]]</f>
         <v>0.92500000000000004</v>
       </c>
       <c r="I15">
@@ -4346,7 +4368,7 @@
         <v>0.35</v>
       </c>
       <c r="M15" s="1">
-        <v>4.4999999999999999E-4</v>
+        <v>3.5E-4</v>
       </c>
       <c r="N15">
         <v>0.12</v>
@@ -4355,6 +4377,58 @@
         <v>10</v>
       </c>
       <c r="P15">
+        <v>0.25</v>
+      </c>
+    </row>
+    <row r="16" spans="1:16" x14ac:dyDescent="0.15">
+      <c r="A16">
+        <v>15</v>
+      </c>
+      <c r="B16">
+        <v>5</v>
+      </c>
+      <c r="C16" t="s">
+        <v>224</v>
+      </c>
+      <c r="D16">
+        <v>0.3</v>
+      </c>
+      <c r="E16">
+        <v>2.5</v>
+      </c>
+      <c r="F16">
+        <v>0.3</v>
+      </c>
+      <c r="G16">
+        <v>18.5</v>
+      </c>
+      <c r="H16">
+        <f>0.05*Tabel10[[#This Row],[Kolom7]]</f>
+        <v>0.92500000000000004</v>
+      </c>
+      <c r="I16">
+        <v>2.5</v>
+      </c>
+      <c r="J16">
+        <v>0.3</v>
+      </c>
+      <c r="K16">
+        <f>2.5*15</f>
+        <v>37.5</v>
+      </c>
+      <c r="L16">
+        <v>0.35</v>
+      </c>
+      <c r="M16" s="1">
+        <v>2.7999999999999998E-4</v>
+      </c>
+      <c r="N16">
+        <v>0.12</v>
+      </c>
+      <c r="O16">
+        <v>10</v>
+      </c>
+      <c r="P16">
         <v>0.25</v>
       </c>
     </row>
@@ -4719,7 +4793,7 @@
         <v>174</v>
       </c>
       <c r="F17" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="I17" s="2"/>
       <c r="J17" s="2"/>

</xml_diff>

<commit_message>
Importeren handmatige frequency lines afgerond
</commit_message>
<xml_diff>
--- a/workspaces/traject_224/input/input.xlsx
+++ b/workspaces/traject_224/input/input.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\CP\git_clones\GeoProb-Pipe\GeoProb-PipeV2\GeoProb-Pipe\workspaces\traject_224\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\CP\git_clones\GeoProb-Pipe\GeoProb-PipeV2\GeoProb-Pipe\workspaces\traject_224\input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{426FC03A-7A33-4DD7-AE89-A1C54559305F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C1F7D0A8-6CA1-4983-8557-2C269E95660C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{E14FA4F5-43AA-4DAE-BCE2-7688F4F5853B}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{E14FA4F5-43AA-4DAE-BCE2-7688F4F5853B}"/>
   </bookViews>
   <sheets>
     <sheet name="Vakken" sheetId="1" r:id="rId1"/>
@@ -657,12 +657,6 @@
     <t>Buitenwaterstand, o.b.v. overschrijdingsfrequentielijn berekend met Pydra in Python</t>
   </si>
   <si>
-    <t>vk0224_0001_1_WA_hm0386</t>
-  </si>
-  <si>
-    <t>vk0224_0002_1_WA_hm0384</t>
-  </si>
-  <si>
     <t>vk0224_0003_1_WA_hm0383</t>
   </si>
   <si>
@@ -712,6 +706,12 @@
   </si>
   <si>
     <t>HA063.+074-RK000.+005</t>
+  </si>
+  <si>
+    <t>vk0224_0002_1_WA_hm0384.csv</t>
+  </si>
+  <si>
+    <t>vk0224_0001_1_WA_hm0386.csv</t>
   </si>
 </sst>
 </file>
@@ -1262,19 +1262,19 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{93C253AA-AAA1-47E5-9332-CA169F978D7A}">
   <dimension ref="A1:I7"/>
-  <sheetFormatPr defaultRowHeight="11.25" x14ac:dyDescent="0.15"/>
+  <sheetFormatPr defaultRowHeight="11.4" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="8.25" customWidth="1"/>
-    <col min="2" max="2" width="36.125" bestFit="1" customWidth="1"/>
-    <col min="3" max="4" width="8.25" customWidth="1"/>
-    <col min="5" max="5" width="16.625" customWidth="1"/>
-    <col min="6" max="6" width="18.25" customWidth="1"/>
-    <col min="7" max="7" width="11.125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="8.19921875" customWidth="1"/>
+    <col min="2" max="2" width="36.09765625" bestFit="1" customWidth="1"/>
+    <col min="3" max="4" width="8.19921875" customWidth="1"/>
+    <col min="5" max="5" width="16.59765625" customWidth="1"/>
+    <col min="6" max="6" width="18.19921875" customWidth="1"/>
+    <col min="7" max="7" width="11.09765625" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="15" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="17.375" customWidth="1"/>
+    <col min="9" max="9" width="17.3984375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" s="5" customFormat="1" x14ac:dyDescent="0.15">
+    <row r="1" spans="1:9" s="5" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A1" s="9" t="s">
         <v>127</v>
       </c>
@@ -1304,12 +1304,12 @@
         <v>c_voorland_stdev</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.15">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A2">
         <v>0</v>
       </c>
       <c r="B2" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="C2">
         <v>0</v>
@@ -1333,12 +1333,12 @@
         <v>0.15</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.15">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="C3">
         <v>446.3</v>
@@ -1362,12 +1362,12 @@
         <v>0.15</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.15">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A4">
         <v>2</v>
       </c>
       <c r="B4" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
       <c r="C4">
         <v>543.4</v>
@@ -1391,12 +1391,12 @@
         <v>0.15</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.15">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A5">
         <v>3</v>
       </c>
       <c r="B5" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="C5">
         <v>750</v>
@@ -1420,12 +1420,12 @@
         <v>0.15</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.15">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A6">
         <v>4</v>
       </c>
       <c r="B6" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="C6">
         <v>844.5</v>
@@ -1449,12 +1449,12 @@
         <v>0.15</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.15">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A7">
         <v>5</v>
       </c>
       <c r="B7" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="C7">
         <v>1121.2</v>
@@ -1486,23 +1486,23 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2AB77777-746E-45C0-BE11-D138C11C003A}">
   <dimension ref="A1:M58"/>
-  <sheetFormatPr defaultRowHeight="11.25" x14ac:dyDescent="0.15"/>
+  <sheetFormatPr defaultRowHeight="11.4" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="14" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="7.375" customWidth="1"/>
-    <col min="3" max="4" width="19.375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="7.3984375" customWidth="1"/>
+    <col min="3" max="4" width="19.3984375" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="15.5" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="8.875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="8.8984375" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="29" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="8.375" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="7.875" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="8.25" customWidth="1"/>
-    <col min="11" max="11" width="23.875" customWidth="1"/>
-    <col min="12" max="12" width="11.875" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="8.625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="8.3984375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="7.8984375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="8.19921875" customWidth="1"/>
+    <col min="11" max="11" width="32.69921875" customWidth="1"/>
+    <col min="12" max="12" width="11.8984375" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="8.59765625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" s="5" customFormat="1" x14ac:dyDescent="0.15">
+    <row r="1" spans="1:13" s="5" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A1" s="9" t="s">
         <v>133</v>
       </c>
@@ -1543,7 +1543,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.15">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A2">
         <v>1</v>
       </c>
@@ -1569,7 +1569,7 @@
         <v>79.8</v>
       </c>
       <c r="K2" t="s">
-        <v>205</v>
+        <v>223</v>
       </c>
       <c r="L2" s="3">
         <v>5.940000057220459</v>
@@ -1578,7 +1578,7 @@
         <v>3.5</v>
       </c>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.15">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>2</v>
       </c>
@@ -1604,7 +1604,7 @@
         <v>32.799999999999997</v>
       </c>
       <c r="K3" t="s">
-        <v>206</v>
+        <v>222</v>
       </c>
       <c r="L3" s="3">
         <v>4.0500001907348633</v>
@@ -1613,7 +1613,7 @@
         <v>3.5</v>
       </c>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.15">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A4">
         <v>3</v>
       </c>
@@ -1639,7 +1639,7 @@
         <v>68.900000000000006</v>
       </c>
       <c r="K4" t="s">
-        <v>206</v>
+        <v>222</v>
       </c>
       <c r="L4" s="3">
         <v>4.0399999618530273</v>
@@ -1648,7 +1648,7 @@
         <v>3.5</v>
       </c>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.15">
+    <row r="5" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A5">
         <v>4</v>
       </c>
@@ -1674,7 +1674,7 @@
         <v>43.4</v>
       </c>
       <c r="K5" t="s">
-        <v>206</v>
+        <v>222</v>
       </c>
       <c r="L5" s="3">
         <v>3.8900001049041748</v>
@@ -1683,7 +1683,7 @@
         <v>3.5</v>
       </c>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.15">
+    <row r="6" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A6">
         <v>5</v>
       </c>
@@ -1709,7 +1709,7 @@
         <v>50.2</v>
       </c>
       <c r="K6" t="s">
-        <v>206</v>
+        <v>222</v>
       </c>
       <c r="L6" s="3">
         <v>3.839999914169312</v>
@@ -1718,7 +1718,7 @@
         <v>3.5</v>
       </c>
     </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.15">
+    <row r="7" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A7">
         <v>6</v>
       </c>
@@ -1744,7 +1744,7 @@
         <v>79.7</v>
       </c>
       <c r="K7" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="L7" s="3">
         <v>4.1100001335144043</v>
@@ -1753,7 +1753,7 @@
         <v>3.5</v>
       </c>
     </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.15">
+    <row r="8" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A8">
         <v>7</v>
       </c>
@@ -1779,7 +1779,7 @@
         <v>54.6</v>
       </c>
       <c r="K8" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="L8" s="3">
         <v>3.9600000381469731</v>
@@ -1788,7 +1788,7 @@
         <v>3.5</v>
       </c>
     </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.15">
+    <row r="9" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A9">
         <v>8</v>
       </c>
@@ -1814,7 +1814,7 @@
         <v>82.6</v>
       </c>
       <c r="K9" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="L9" s="3">
         <v>3.8199999332427979</v>
@@ -1823,7 +1823,7 @@
         <v>3.5</v>
       </c>
     </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.15">
+    <row r="10" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A10">
         <v>9</v>
       </c>
@@ -1849,7 +1849,7 @@
         <v>71</v>
       </c>
       <c r="K10" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="L10" s="3">
         <v>2.7100000381469731</v>
@@ -1858,7 +1858,7 @@
         <v>3.5</v>
       </c>
     </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.15">
+    <row r="11" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A11">
         <v>10</v>
       </c>
@@ -1884,7 +1884,7 @@
         <v>38.299999999999997</v>
       </c>
       <c r="K11" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="L11" s="3">
         <v>3.9900000095367432</v>
@@ -1893,7 +1893,7 @@
         <v>3.5</v>
       </c>
     </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.15">
+    <row r="12" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A12">
         <v>11</v>
       </c>
@@ -1919,7 +1919,7 @@
         <v>77.3</v>
       </c>
       <c r="K12" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="L12" s="3">
         <v>2.630000114440918</v>
@@ -1928,7 +1928,7 @@
         <v>3.5</v>
       </c>
     </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.15">
+    <row r="13" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A13">
         <v>12</v>
       </c>
@@ -1954,7 +1954,7 @@
         <v>44.6</v>
       </c>
       <c r="K13" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="L13" s="3">
         <v>3.9800000190734859</v>
@@ -1963,7 +1963,7 @@
         <v>3.5</v>
       </c>
     </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.15">
+    <row r="14" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A14">
         <v>13</v>
       </c>
@@ -1989,7 +1989,7 @@
         <v>80.099999999999994</v>
       </c>
       <c r="K14" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="L14" s="3">
         <v>2.6700000762939449</v>
@@ -1998,7 +1998,7 @@
         <v>3.5</v>
       </c>
     </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.15">
+    <row r="15" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A15">
         <v>15</v>
       </c>
@@ -2024,7 +2024,7 @@
         <v>15.4</v>
       </c>
       <c r="K15" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="L15" s="3">
         <v>6.5900001525878906</v>
@@ -2033,7 +2033,7 @@
         <v>3.5</v>
       </c>
     </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.15">
+    <row r="16" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A16">
         <v>16</v>
       </c>
@@ -2059,7 +2059,7 @@
         <v>60.9</v>
       </c>
       <c r="K16" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="L16" s="3">
         <v>4.440000057220459</v>
@@ -2068,7 +2068,7 @@
         <v>3.5</v>
       </c>
     </row>
-    <row r="17" spans="1:13" x14ac:dyDescent="0.15">
+    <row r="17" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A17">
         <v>17</v>
       </c>
@@ -2094,7 +2094,7 @@
         <v>87.7</v>
       </c>
       <c r="K17" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="L17" s="3">
         <v>3.0499999523162842</v>
@@ -2103,7 +2103,7 @@
         <v>3.5</v>
       </c>
     </row>
-    <row r="18" spans="1:13" x14ac:dyDescent="0.15">
+    <row r="18" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A18">
         <v>18</v>
       </c>
@@ -2129,7 +2129,7 @@
         <v>87.6</v>
       </c>
       <c r="K18" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="L18" s="3">
         <v>2.7400000095367432</v>
@@ -2138,7 +2138,7 @@
         <v>3.5</v>
       </c>
     </row>
-    <row r="19" spans="1:13" x14ac:dyDescent="0.15">
+    <row r="19" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A19">
         <v>19</v>
       </c>
@@ -2164,7 +2164,7 @@
         <v>89.1</v>
       </c>
       <c r="K19" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="L19" s="3">
         <v>3.7999999523162842</v>
@@ -2173,7 +2173,7 @@
         <v>3.5</v>
       </c>
     </row>
-    <row r="20" spans="1:13" x14ac:dyDescent="0.15">
+    <row r="20" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A20">
         <v>20</v>
       </c>
@@ -2199,7 +2199,7 @@
         <v>77.3</v>
       </c>
       <c r="K20" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="L20" s="3">
         <v>4.059999942779541</v>
@@ -2208,7 +2208,7 @@
         <v>3.5</v>
       </c>
     </row>
-    <row r="21" spans="1:13" x14ac:dyDescent="0.15">
+    <row r="21" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A21">
         <v>21</v>
       </c>
@@ -2234,7 +2234,7 @@
         <v>71.2</v>
       </c>
       <c r="K21" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="L21" s="3">
         <v>5.809999942779541</v>
@@ -2243,7 +2243,7 @@
         <v>3.5</v>
       </c>
     </row>
-    <row r="22" spans="1:13" x14ac:dyDescent="0.15">
+    <row r="22" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A22">
         <v>22</v>
       </c>
@@ -2269,7 +2269,7 @@
         <v>77.400000000000006</v>
       </c>
       <c r="K22" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="L22" s="3">
         <v>6.0300002098083496</v>
@@ -2278,7 +2278,7 @@
         <v>3.5</v>
       </c>
     </row>
-    <row r="23" spans="1:13" x14ac:dyDescent="0.15">
+    <row r="23" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A23">
         <v>23</v>
       </c>
@@ -2304,7 +2304,7 @@
         <v>71.8</v>
       </c>
       <c r="K23" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="L23" s="3">
         <v>5.4800000190734863</v>
@@ -2313,7 +2313,7 @@
         <v>3.5</v>
       </c>
     </row>
-    <row r="24" spans="1:13" x14ac:dyDescent="0.15">
+    <row r="24" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A24">
         <v>24</v>
       </c>
@@ -2339,7 +2339,7 @@
         <v>72.3</v>
       </c>
       <c r="K24" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="L24" s="3">
         <v>5.4899997711181641</v>
@@ -2348,7 +2348,7 @@
         <v>3.5</v>
       </c>
     </row>
-    <row r="25" spans="1:13" x14ac:dyDescent="0.15">
+    <row r="25" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A25">
         <v>25</v>
       </c>
@@ -2374,7 +2374,7 @@
         <v>76</v>
       </c>
       <c r="K25" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="L25" s="3">
         <v>5.5799999237060547</v>
@@ -2383,7 +2383,7 @@
         <v>3.5</v>
       </c>
     </row>
-    <row r="26" spans="1:13" x14ac:dyDescent="0.15">
+    <row r="26" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A26">
         <v>26</v>
       </c>
@@ -2409,7 +2409,7 @@
         <v>79.8</v>
       </c>
       <c r="K26" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="L26" s="3">
         <v>4.3499999046325684</v>
@@ -2418,7 +2418,7 @@
         <v>3.5</v>
       </c>
     </row>
-    <row r="27" spans="1:13" x14ac:dyDescent="0.15">
+    <row r="27" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A27">
         <v>27</v>
       </c>
@@ -2444,7 +2444,7 @@
         <v>38.4</v>
       </c>
       <c r="K27" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="L27" s="3">
         <v>4.7300000190734863</v>
@@ -2453,7 +2453,7 @@
         <v>3.5</v>
       </c>
     </row>
-    <row r="28" spans="1:13" x14ac:dyDescent="0.15">
+    <row r="28" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A28">
         <v>28</v>
       </c>
@@ -2479,7 +2479,7 @@
         <v>62.3</v>
       </c>
       <c r="K28" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="L28" s="3">
         <v>5.5300002098083496</v>
@@ -2488,7 +2488,7 @@
         <v>3.5</v>
       </c>
     </row>
-    <row r="29" spans="1:13" x14ac:dyDescent="0.15">
+    <row r="29" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A29">
         <v>29</v>
       </c>
@@ -2514,7 +2514,7 @@
         <v>38.299999999999997</v>
       </c>
       <c r="K29" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="L29" s="3">
         <v>5.619999885559082</v>
@@ -2523,7 +2523,7 @@
         <v>3.5</v>
       </c>
     </row>
-    <row r="30" spans="1:13" x14ac:dyDescent="0.15">
+    <row r="30" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A30">
         <v>30</v>
       </c>
@@ -2549,7 +2549,7 @@
         <v>89.6</v>
       </c>
       <c r="K30" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="L30" s="3">
         <v>5.5900001525878906</v>
@@ -2558,7 +2558,7 @@
         <v>3.5</v>
       </c>
     </row>
-    <row r="31" spans="1:13" x14ac:dyDescent="0.15">
+    <row r="31" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A31">
         <v>31</v>
       </c>
@@ -2584,7 +2584,7 @@
         <v>77.2</v>
       </c>
       <c r="K31" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="L31" s="3">
         <v>5.7399997711181641</v>
@@ -2593,7 +2593,7 @@
         <v>3.5</v>
       </c>
     </row>
-    <row r="32" spans="1:13" x14ac:dyDescent="0.15">
+    <row r="32" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A32">
         <v>32</v>
       </c>
@@ -2619,7 +2619,7 @@
         <v>27.9</v>
       </c>
       <c r="K32" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="L32" s="3">
         <v>5.7699999809265137</v>
@@ -2628,7 +2628,7 @@
         <v>3.5</v>
       </c>
     </row>
-    <row r="33" spans="1:13" x14ac:dyDescent="0.15">
+    <row r="33" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A33">
         <v>33</v>
       </c>
@@ -2654,7 +2654,7 @@
         <v>66.5</v>
       </c>
       <c r="K33" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="L33" s="3">
         <v>5.8400001525878906</v>
@@ -2663,7 +2663,7 @@
         <v>3.5</v>
       </c>
     </row>
-    <row r="34" spans="1:13" x14ac:dyDescent="0.15">
+    <row r="34" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A34">
         <v>34</v>
       </c>
@@ -2689,7 +2689,7 @@
         <v>63.8</v>
       </c>
       <c r="K34" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="L34" s="3">
         <v>5.8400001525878906</v>
@@ -2698,7 +2698,7 @@
         <v>3.5</v>
       </c>
     </row>
-    <row r="35" spans="1:13" x14ac:dyDescent="0.15">
+    <row r="35" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A35">
         <v>35</v>
       </c>
@@ -2724,7 +2724,7 @@
         <v>24.7</v>
       </c>
       <c r="K35" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="L35" s="3">
         <v>5.9200000762939453</v>
@@ -2733,7 +2733,7 @@
         <v>3.5</v>
       </c>
     </row>
-    <row r="36" spans="1:13" x14ac:dyDescent="0.15">
+    <row r="36" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A36">
         <v>36</v>
       </c>
@@ -2759,7 +2759,7 @@
         <v>43.4</v>
       </c>
       <c r="K36" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="L36" s="3">
         <v>5.869999885559082</v>
@@ -2768,7 +2768,7 @@
         <v>3.5</v>
       </c>
     </row>
-    <row r="37" spans="1:13" x14ac:dyDescent="0.15">
+    <row r="37" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A37">
         <v>37</v>
       </c>
@@ -2794,7 +2794,7 @@
         <v>24.3</v>
       </c>
       <c r="K37" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="L37" s="3">
         <v>5.869999885559082</v>
@@ -2803,7 +2803,7 @@
         <v>3.5</v>
       </c>
     </row>
-    <row r="38" spans="1:13" x14ac:dyDescent="0.15">
+    <row r="38" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A38">
         <v>38</v>
       </c>
@@ -2829,7 +2829,7 @@
         <v>25.2</v>
       </c>
       <c r="K38" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="L38" s="3">
         <v>5.880000114440918</v>
@@ -2838,7 +2838,7 @@
         <v>3.5</v>
       </c>
     </row>
-    <row r="39" spans="1:13" x14ac:dyDescent="0.15">
+    <row r="39" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A39">
         <v>39</v>
       </c>
@@ -2864,7 +2864,7 @@
         <v>52.6</v>
       </c>
       <c r="K39" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="L39" s="3">
         <v>5.4200000762939453</v>
@@ -2873,7 +2873,7 @@
         <v>3.5</v>
       </c>
     </row>
-    <row r="40" spans="1:13" x14ac:dyDescent="0.15">
+    <row r="40" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A40">
         <v>40</v>
       </c>
@@ -2899,7 +2899,7 @@
         <v>10.9</v>
       </c>
       <c r="K40" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="L40" s="3">
         <v>6.3600001335144043</v>
@@ -2908,7 +2908,7 @@
         <v>3.5</v>
       </c>
     </row>
-    <row r="41" spans="1:13" x14ac:dyDescent="0.15">
+    <row r="41" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A41">
         <v>41</v>
       </c>
@@ -2934,7 +2934,7 @@
         <v>63.7</v>
       </c>
       <c r="K41" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="L41" s="3">
         <v>5.5900001525878906</v>
@@ -2943,7 +2943,7 @@
         <v>3.5</v>
       </c>
     </row>
-    <row r="42" spans="1:13" x14ac:dyDescent="0.15">
+    <row r="42" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A42">
         <v>42</v>
       </c>
@@ -2969,7 +2969,7 @@
         <v>63.2</v>
       </c>
       <c r="K42" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="L42" s="3">
         <v>5.5</v>
@@ -2978,7 +2978,7 @@
         <v>3.5</v>
       </c>
     </row>
-    <row r="43" spans="1:13" x14ac:dyDescent="0.15">
+    <row r="43" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A43">
         <v>43</v>
       </c>
@@ -3004,7 +3004,7 @@
         <v>35.6</v>
       </c>
       <c r="K43" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="L43" s="3">
         <v>6.070000171661377</v>
@@ -3013,7 +3013,7 @@
         <v>3.5</v>
       </c>
     </row>
-    <row r="44" spans="1:13" x14ac:dyDescent="0.15">
+    <row r="44" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A44">
         <v>44</v>
       </c>
@@ -3039,7 +3039,7 @@
         <v>83.7</v>
       </c>
       <c r="K44" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="L44" s="3">
         <v>5.2800002098083496</v>
@@ -3048,7 +3048,7 @@
         <v>3.5</v>
       </c>
     </row>
-    <row r="45" spans="1:13" x14ac:dyDescent="0.15">
+    <row r="45" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A45">
         <v>45</v>
       </c>
@@ -3074,7 +3074,7 @@
         <v>71.099999999999994</v>
       </c>
       <c r="K45" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="L45" s="3">
         <v>5.1599998474121094</v>
@@ -3083,7 +3083,7 @@
         <v>3.5</v>
       </c>
     </row>
-    <row r="46" spans="1:13" x14ac:dyDescent="0.15">
+    <row r="46" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A46">
         <v>46</v>
       </c>
@@ -3109,7 +3109,7 @@
         <v>15</v>
       </c>
       <c r="K46" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="L46" s="3">
         <v>6.0799999237060547</v>
@@ -3118,7 +3118,7 @@
         <v>3.5</v>
       </c>
     </row>
-    <row r="47" spans="1:13" x14ac:dyDescent="0.15">
+    <row r="47" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A47">
         <v>47</v>
       </c>
@@ -3144,7 +3144,7 @@
         <v>76.599999999999994</v>
       </c>
       <c r="K47" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="L47" s="3">
         <v>3.9900000095367432</v>
@@ -3153,7 +3153,7 @@
         <v>3.5</v>
       </c>
     </row>
-    <row r="48" spans="1:13" x14ac:dyDescent="0.15">
+    <row r="48" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A48">
         <v>48</v>
       </c>
@@ -3179,7 +3179,7 @@
         <v>83.1</v>
       </c>
       <c r="K48" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="L48" s="3">
         <v>3.9600000381469731</v>
@@ -3188,7 +3188,7 @@
         <v>3.5</v>
       </c>
     </row>
-    <row r="49" spans="1:13" x14ac:dyDescent="0.15">
+    <row r="49" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A49">
         <v>49</v>
       </c>
@@ -3214,7 +3214,7 @@
         <v>78.900000000000006</v>
       </c>
       <c r="K49" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="L49" s="3">
         <v>5.0399999618530273</v>
@@ -3223,7 +3223,7 @@
         <v>3.5</v>
       </c>
     </row>
-    <row r="50" spans="1:13" x14ac:dyDescent="0.15">
+    <row r="50" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A50">
         <v>50</v>
       </c>
@@ -3249,7 +3249,7 @@
         <v>46.4</v>
       </c>
       <c r="K50" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="L50" s="3">
         <v>5.0199999809265137</v>
@@ -3258,7 +3258,7 @@
         <v>3.5</v>
       </c>
     </row>
-    <row r="51" spans="1:13" x14ac:dyDescent="0.15">
+    <row r="51" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A51">
         <v>51</v>
       </c>
@@ -3284,7 +3284,7 @@
         <v>77.400000000000006</v>
       </c>
       <c r="K51" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="L51" s="3">
         <v>5.0399999618530273</v>
@@ -3293,7 +3293,7 @@
         <v>3.5</v>
       </c>
     </row>
-    <row r="52" spans="1:13" x14ac:dyDescent="0.15">
+    <row r="52" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A52">
         <v>52</v>
       </c>
@@ -3319,7 +3319,7 @@
         <v>49.7</v>
       </c>
       <c r="K52" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="L52" s="3">
         <v>5.0199999809265137</v>
@@ -3328,7 +3328,7 @@
         <v>3.5</v>
       </c>
     </row>
-    <row r="53" spans="1:13" x14ac:dyDescent="0.15">
+    <row r="53" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A53">
         <v>53</v>
       </c>
@@ -3354,7 +3354,7 @@
         <v>27.6</v>
       </c>
       <c r="K53" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="L53" s="3">
         <v>5.0100002288818359</v>
@@ -3363,7 +3363,7 @@
         <v>3.5</v>
       </c>
     </row>
-    <row r="54" spans="1:13" x14ac:dyDescent="0.15">
+    <row r="54" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A54">
         <v>54</v>
       </c>
@@ -3389,7 +3389,7 @@
         <v>75.599999999999994</v>
       </c>
       <c r="K54" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="L54" s="3">
         <v>4.9200000762939453</v>
@@ -3398,7 +3398,7 @@
         <v>3.5</v>
       </c>
     </row>
-    <row r="55" spans="1:13" x14ac:dyDescent="0.15">
+    <row r="55" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A55">
         <v>55</v>
       </c>
@@ -3424,7 +3424,7 @@
         <v>47.4</v>
       </c>
       <c r="K55" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="L55" s="3">
         <v>4.9800000190734863</v>
@@ -3433,7 +3433,7 @@
         <v>3.5</v>
       </c>
     </row>
-    <row r="56" spans="1:13" x14ac:dyDescent="0.15">
+    <row r="56" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A56">
         <v>56</v>
       </c>
@@ -3459,7 +3459,7 @@
         <v>25.9</v>
       </c>
       <c r="K56" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="L56" s="3">
         <v>6.179999828338623</v>
@@ -3468,7 +3468,7 @@
         <v>3.5</v>
       </c>
     </row>
-    <row r="57" spans="1:13" x14ac:dyDescent="0.15">
+    <row r="57" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A57">
         <v>57</v>
       </c>
@@ -3494,7 +3494,7 @@
         <v>77.599999999999994</v>
       </c>
       <c r="K57" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="L57" s="3">
         <v>5.4699997901916504</v>
@@ -3503,7 +3503,7 @@
         <v>3.5</v>
       </c>
     </row>
-    <row r="58" spans="1:13" x14ac:dyDescent="0.15">
+    <row r="58" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A58">
         <v>58</v>
       </c>
@@ -3529,7 +3529,7 @@
         <v>55.1</v>
       </c>
       <c r="K58" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="L58" s="3">
         <v>4.9600000381469727</v>
@@ -3550,24 +3550,24 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A3ED9FF6-8968-4FA6-BAEC-B95365AA2886}">
   <dimension ref="A1:P15"/>
-  <sheetFormatPr defaultRowHeight="11.25" x14ac:dyDescent="0.15"/>
+  <sheetFormatPr defaultRowHeight="11.4" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="20.75" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="6.75" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="21.75" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="20.69921875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="6.69921875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="21.69921875" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="21" bestFit="1" customWidth="1"/>
-    <col min="5" max="6" width="13.875" bestFit="1" customWidth="1"/>
-    <col min="7" max="8" width="23.125" bestFit="1" customWidth="1"/>
-    <col min="9" max="10" width="11.625" bestFit="1" customWidth="1"/>
+    <col min="5" max="6" width="13.8984375" bestFit="1" customWidth="1"/>
+    <col min="7" max="8" width="23.09765625" bestFit="1" customWidth="1"/>
+    <col min="9" max="10" width="11.59765625" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="12.5" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="11.375" customWidth="1"/>
-    <col min="13" max="13" width="9.25" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.25" customWidth="1"/>
+    <col min="12" max="12" width="11.3984375" customWidth="1"/>
+    <col min="13" max="13" width="9.19921875" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="9.19921875" customWidth="1"/>
     <col min="15" max="15" width="16.5" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="16.625" customWidth="1"/>
+    <col min="16" max="16" width="16.59765625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" s="5" customFormat="1" x14ac:dyDescent="0.15">
+    <row r="1" spans="1:16" s="5" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A1" s="9" t="s">
         <v>136</v>
       </c>
@@ -3623,7 +3623,7 @@
         <v>c_achterland_vc</v>
       </c>
     </row>
-    <row r="2" spans="1:16" x14ac:dyDescent="0.15">
+    <row r="2" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A2">
         <v>1</v>
       </c>
@@ -3673,7 +3673,7 @@
         <v>0.25</v>
       </c>
     </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.15">
+    <row r="3" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>2</v>
       </c>
@@ -3723,7 +3723,7 @@
         <v>0.25</v>
       </c>
     </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.15">
+    <row r="4" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A4">
         <v>1</v>
       </c>
@@ -3773,7 +3773,7 @@
         <v>0.25</v>
       </c>
     </row>
-    <row r="5" spans="1:16" x14ac:dyDescent="0.15">
+    <row r="5" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A5">
         <v>2</v>
       </c>
@@ -3823,7 +3823,7 @@
         <v>0.25</v>
       </c>
     </row>
-    <row r="6" spans="1:16" x14ac:dyDescent="0.15">
+    <row r="6" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A6">
         <v>3</v>
       </c>
@@ -3873,7 +3873,7 @@
         <v>0.25</v>
       </c>
     </row>
-    <row r="7" spans="1:16" x14ac:dyDescent="0.15">
+    <row r="7" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A7">
         <v>4</v>
       </c>
@@ -3923,7 +3923,7 @@
         <v>0.25</v>
       </c>
     </row>
-    <row r="8" spans="1:16" x14ac:dyDescent="0.15">
+    <row r="8" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A8">
         <v>5</v>
       </c>
@@ -3973,7 +3973,7 @@
         <v>0.25</v>
       </c>
     </row>
-    <row r="9" spans="1:16" x14ac:dyDescent="0.15">
+    <row r="9" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A9">
         <v>6</v>
       </c>
@@ -4023,7 +4023,7 @@
         <v>0.25</v>
       </c>
     </row>
-    <row r="10" spans="1:16" x14ac:dyDescent="0.15">
+    <row r="10" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A10">
         <v>7</v>
       </c>
@@ -4073,7 +4073,7 @@
         <v>0.25</v>
       </c>
     </row>
-    <row r="11" spans="1:16" x14ac:dyDescent="0.15">
+    <row r="11" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A11">
         <v>8</v>
       </c>
@@ -4123,7 +4123,7 @@
         <v>0.25</v>
       </c>
     </row>
-    <row r="12" spans="1:16" x14ac:dyDescent="0.15">
+    <row r="12" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A12">
         <v>9</v>
       </c>
@@ -4173,7 +4173,7 @@
         <v>0.25</v>
       </c>
     </row>
-    <row r="13" spans="1:16" x14ac:dyDescent="0.15">
+    <row r="13" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A13">
         <v>10</v>
       </c>
@@ -4223,7 +4223,7 @@
         <v>0.25</v>
       </c>
     </row>
-    <row r="14" spans="1:16" x14ac:dyDescent="0.15">
+    <row r="14" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A14">
         <v>11</v>
       </c>
@@ -4273,7 +4273,7 @@
         <v>0.25</v>
       </c>
     </row>
-    <row r="15" spans="1:16" x14ac:dyDescent="0.15">
+    <row r="15" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A15">
         <v>12</v>
       </c>
@@ -4334,25 +4334,25 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B9B7A8CE-63DA-4EEA-9A88-5E62FD2B5E40}">
   <dimension ref="A1:P69"/>
-  <sheetFormatPr defaultRowHeight="11.25" x14ac:dyDescent="0.15"/>
+  <sheetFormatPr defaultRowHeight="11.4" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="22.5" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="71.125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="22.375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="23.875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="29.625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="19.25" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="71.09765625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22.3984375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="23.8984375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="29.59765625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="19.19921875" bestFit="1" customWidth="1"/>
     <col min="7" max="8" width="23" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="17.375" bestFit="1" customWidth="1"/>
-    <col min="10" max="11" width="17.25" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="17.3984375" bestFit="1" customWidth="1"/>
+    <col min="10" max="11" width="17.19921875" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="18" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.25" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="14.25" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="13.19921875" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="14.19921875" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="14" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="51.125" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="51.09765625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" s="5" customFormat="1" x14ac:dyDescent="0.15">
+    <row r="1" spans="1:16" s="5" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A1" s="4" t="s">
         <v>200</v>
       </c>
@@ -4402,7 +4402,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="2" spans="1:16" x14ac:dyDescent="0.15">
+    <row r="2" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>127</v>
       </c>
@@ -4419,7 +4419,7 @@
       <c r="J2" s="2"/>
       <c r="K2" s="2"/>
     </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.15">
+    <row r="3" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>128</v>
       </c>
@@ -4436,7 +4436,7 @@
       <c r="J3" s="2"/>
       <c r="K3" s="2"/>
     </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.15">
+    <row r="4" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>0</v>
       </c>
@@ -4451,7 +4451,7 @@
       <c r="J4" s="2"/>
       <c r="K4" s="2"/>
     </row>
-    <row r="5" spans="1:16" x14ac:dyDescent="0.15">
+    <row r="5" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>1</v>
       </c>
@@ -4466,7 +4466,7 @@
       <c r="J5" s="2"/>
       <c r="K5" s="2"/>
     </row>
-    <row r="6" spans="1:16" x14ac:dyDescent="0.15">
+    <row r="6" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>129</v>
       </c>
@@ -4483,7 +4483,7 @@
       <c r="J6" s="2"/>
       <c r="K6" s="2"/>
     </row>
-    <row r="7" spans="1:16" x14ac:dyDescent="0.15">
+    <row r="7" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>133</v>
       </c>
@@ -4500,7 +4500,7 @@
       <c r="J7" s="2"/>
       <c r="K7" s="2"/>
     </row>
-    <row r="8" spans="1:16" x14ac:dyDescent="0.15">
+    <row r="8" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>134</v>
       </c>
@@ -4517,7 +4517,7 @@
       <c r="J8" s="2"/>
       <c r="K8" s="2"/>
     </row>
-    <row r="9" spans="1:16" x14ac:dyDescent="0.15">
+    <row r="9" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>135</v>
       </c>
@@ -4534,7 +4534,7 @@
       <c r="J9" s="2"/>
       <c r="K9" s="2"/>
     </row>
-    <row r="10" spans="1:16" x14ac:dyDescent="0.15">
+    <row r="10" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>130</v>
       </c>
@@ -4551,7 +4551,7 @@
       <c r="J10" s="2"/>
       <c r="K10" s="2"/>
     </row>
-    <row r="11" spans="1:16" x14ac:dyDescent="0.15">
+    <row r="11" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>131</v>
       </c>
@@ -4566,7 +4566,7 @@
       <c r="J11" s="2"/>
       <c r="K11" s="2"/>
     </row>
-    <row r="12" spans="1:16" x14ac:dyDescent="0.15">
+    <row r="12" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>132</v>
       </c>
@@ -4581,7 +4581,7 @@
       <c r="J12" s="2"/>
       <c r="K12" s="2"/>
     </row>
-    <row r="13" spans="1:16" x14ac:dyDescent="0.15">
+    <row r="13" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>136</v>
       </c>
@@ -4598,7 +4598,7 @@
       <c r="J13" s="2"/>
       <c r="K13" s="2"/>
     </row>
-    <row r="14" spans="1:16" x14ac:dyDescent="0.15">
+    <row r="14" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>137</v>
       </c>
@@ -4615,7 +4615,7 @@
       <c r="J14" s="2"/>
       <c r="K14" s="2"/>
     </row>
-    <row r="15" spans="1:16" x14ac:dyDescent="0.15">
+    <row r="15" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>138</v>
       </c>
@@ -4639,7 +4639,7 @@
       </c>
       <c r="K15" s="2"/>
     </row>
-    <row r="16" spans="1:16" x14ac:dyDescent="0.15">
+    <row r="16" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>52</v>
       </c>
@@ -4667,7 +4667,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="17" spans="1:16" x14ac:dyDescent="0.15">
+    <row r="17" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>49</v>
       </c>
@@ -4698,7 +4698,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="18" spans="1:16" x14ac:dyDescent="0.15">
+    <row r="18" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>41</v>
       </c>
@@ -4730,7 +4730,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="19" spans="1:16" x14ac:dyDescent="0.15">
+    <row r="19" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>46</v>
       </c>
@@ -4765,7 +4765,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="20" spans="1:16" x14ac:dyDescent="0.15">
+    <row r="20" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>29</v>
       </c>
@@ -4794,7 +4794,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="21" spans="1:16" x14ac:dyDescent="0.15">
+    <row r="21" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>38</v>
       </c>
@@ -4835,7 +4835,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="22" spans="1:16" x14ac:dyDescent="0.15">
+    <row r="22" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>3</v>
       </c>
@@ -4870,7 +4870,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="23" spans="1:16" x14ac:dyDescent="0.15">
+    <row r="23" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
         <v>8</v>
       </c>
@@ -4903,7 +4903,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="24" spans="1:16" x14ac:dyDescent="0.15">
+    <row r="24" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
         <v>7</v>
       </c>
@@ -4939,7 +4939,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="25" spans="1:16" x14ac:dyDescent="0.15">
+    <row r="25" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
         <v>6</v>
       </c>
@@ -4977,7 +4977,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="26" spans="1:16" x14ac:dyDescent="0.15">
+    <row r="26" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
         <v>2</v>
       </c>
@@ -4999,7 +4999,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="27" spans="1:16" x14ac:dyDescent="0.15">
+    <row r="27" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
         <v>10</v>
       </c>
@@ -5028,7 +5028,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="28" spans="1:16" x14ac:dyDescent="0.15">
+    <row r="28" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
         <v>11</v>
       </c>
@@ -5062,7 +5062,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="29" spans="1:16" x14ac:dyDescent="0.15">
+    <row r="29" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
         <v>26</v>
       </c>
@@ -5094,7 +5094,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="30" spans="1:16" x14ac:dyDescent="0.15">
+    <row r="30" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
         <v>78</v>
       </c>
@@ -5123,7 +5123,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="31" spans="1:16" x14ac:dyDescent="0.15">
+    <row r="31" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
         <v>65</v>
       </c>
@@ -5148,7 +5148,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="32" spans="1:16" x14ac:dyDescent="0.15">
+    <row r="32" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
         <v>80</v>
       </c>
@@ -5176,7 +5176,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="33" spans="1:16" x14ac:dyDescent="0.15">
+    <row r="33" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
         <v>85</v>
       </c>
@@ -5205,7 +5205,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="34" spans="1:16" x14ac:dyDescent="0.15">
+    <row r="34" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
         <v>36</v>
       </c>
@@ -5230,7 +5230,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="35" spans="1:16" x14ac:dyDescent="0.15">
+    <row r="35" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
         <v>125</v>
       </c>
@@ -5253,7 +5253,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="36" spans="1:16" x14ac:dyDescent="0.15">
+    <row r="36" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
         <v>60</v>
       </c>
@@ -5287,7 +5287,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="37" spans="1:16" x14ac:dyDescent="0.15">
+    <row r="37" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
         <v>121</v>
       </c>
@@ -5316,7 +5316,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="38" spans="1:16" x14ac:dyDescent="0.15">
+    <row r="38" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
         <v>123</v>
       </c>
@@ -5345,7 +5345,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="39" spans="1:16" x14ac:dyDescent="0.15">
+    <row r="39" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
         <v>63</v>
       </c>
@@ -5374,7 +5374,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="40" spans="1:16" x14ac:dyDescent="0.15">
+    <row r="40" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
         <v>75</v>
       </c>
@@ -5403,7 +5403,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="41" spans="1:16" x14ac:dyDescent="0.15">
+    <row r="41" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
         <v>83</v>
       </c>
@@ -5432,7 +5432,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="42" spans="1:16" x14ac:dyDescent="0.15">
+    <row r="42" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
         <v>57</v>
       </c>
@@ -5466,7 +5466,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="43" spans="1:16" x14ac:dyDescent="0.15">
+    <row r="43" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
         <v>58</v>
       </c>
@@ -5500,7 +5500,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="44" spans="1:16" x14ac:dyDescent="0.15">
+    <row r="44" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
         <v>54</v>
       </c>
@@ -5534,7 +5534,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="45" spans="1:16" x14ac:dyDescent="0.15">
+    <row r="45" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
         <v>9</v>
       </c>
@@ -5559,7 +5559,7 @@
         <v>203</v>
       </c>
     </row>
-    <row r="46" spans="1:16" x14ac:dyDescent="0.15">
+    <row r="46" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
         <v>32</v>
       </c>
@@ -5581,7 +5581,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="47" spans="1:16" x14ac:dyDescent="0.15">
+    <row r="47" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
         <v>34</v>
       </c>
@@ -5603,7 +5603,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="48" spans="1:16" x14ac:dyDescent="0.15">
+    <row r="48" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
         <v>93</v>
       </c>
@@ -5625,7 +5625,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="49" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="49" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
         <v>89</v>
       </c>
@@ -5647,7 +5647,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="50" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="50" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
         <v>87</v>
       </c>
@@ -5669,7 +5669,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="51" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="51" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
         <v>117</v>
       </c>
@@ -5691,7 +5691,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="52" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="52" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
         <v>119</v>
       </c>
@@ -5713,7 +5713,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="53" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="53" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
         <v>115</v>
       </c>
@@ -5735,7 +5735,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="54" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="54" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
         <v>70</v>
       </c>
@@ -5757,7 +5757,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="55" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="55" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
         <v>91</v>
       </c>
@@ -5779,7 +5779,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="56" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="56" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
         <v>43</v>
       </c>
@@ -5798,7 +5798,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="57" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="57" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
         <v>105</v>
       </c>
@@ -5820,7 +5820,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="58" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="58" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
         <v>73</v>
       </c>
@@ -5842,7 +5842,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="59" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="59" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
         <v>103</v>
       </c>
@@ -5864,7 +5864,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="60" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="60" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A60" t="s">
         <v>109</v>
       </c>
@@ -5886,7 +5886,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="61" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="61" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A61" t="s">
         <v>107</v>
       </c>
@@ -5908,7 +5908,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="62" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="62" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A62" t="s">
         <v>69</v>
       </c>
@@ -5936,7 +5936,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="63" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="63" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A63" t="s">
         <v>67</v>
       </c>
@@ -5958,7 +5958,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="64" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="64" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A64" t="s">
         <v>113</v>
       </c>
@@ -5980,7 +5980,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="65" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="65" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A65" t="s">
         <v>111</v>
       </c>
@@ -6002,7 +6002,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="66" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="66" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A66" t="s">
         <v>101</v>
       </c>
@@ -6030,7 +6030,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="67" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="67" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A67" t="s">
         <v>97</v>
       </c>
@@ -6052,7 +6052,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="68" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="68" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A68" t="s">
         <v>99</v>
       </c>
@@ -6074,7 +6074,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="69" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="69" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A69" t="s">
         <v>95</v>
       </c>
@@ -6139,13 +6139,13 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7F7FD5E8-359B-4F56-B38E-FCA72B85D698}">
   <dimension ref="A1:C6"/>
-  <sheetFormatPr defaultColWidth="8.75" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.69921875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="23.125" style="7" bestFit="1" customWidth="1"/>
-    <col min="2" max="16384" width="8.75" style="7"/>
+    <col min="1" max="1" width="23.09765625" style="7" bestFit="1" customWidth="1"/>
+    <col min="2" max="16384" width="8.69921875" style="7"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="8" t="s">
         <v>187</v>
       </c>
@@ -6156,7 +6156,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" s="7" t="s">
         <v>184</v>
       </c>
@@ -6167,7 +6167,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" s="7" t="s">
         <v>181</v>
       </c>
@@ -6178,7 +6178,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" s="7" t="s">
         <v>180</v>
       </c>
@@ -6189,7 +6189,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" s="7" t="s">
         <v>178</v>
       </c>
@@ -6200,7 +6200,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" s="7" t="s">
         <v>176</v>
       </c>

</xml_diff>